<commit_message>
Rebrand to individual collective-housing dashboard with new map, logo, and 4 pillars
- Title: "لوحة معلومات السكن الجماعي للأفراد بمدينة الرياض"; deputy renamed
  to وكالة التنمية الحضرية across UI, workbook, and README
- Riyadh map redrawn to match the official sector map layout (north
  center-left, large east, small center, west, large south); facility
  and hotspot coordinates resampled inside the new polygons with a
  deterministic point-in-polygon clamp; sector labels now render above
  the dots with a halo
- Rail logo replaced with a vector Riyadh Municipality roundel (Masmak
  fortress + الرياض band)
- KPI gauges reduced to a single gauge each (removed the overlay target
  pointer that read as a second clock hand)
- Strategic pillars consolidated from 7 to 4 (الأنظمة والتشريعات،
  النموذج الحضري، الاستثمار والقطاع الخاص، الرقابة) with the same 28
  initiatives regrouped 7 per pillar; pillar grid and copy updated
</commit_message>
<xml_diff>
--- a/riyadh-labor-accommodation/labor_accommodation_data.xlsx
+++ b/riyadh-labor-accommodation/labor_accommodation_data.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>أمانة منطقة الرياض — وكالة سكن العمالة (بيانات تجريبية لأغراض العرض)</t>
+          <t>أمانة منطقة الرياض — وكالة التنمية الحضرية (بيانات تجريبية لأغراض العرض)</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28 مبادرة على 7 ركائز، 14 مؤشر أداء، وتوقعات 12 شهراً بثلاثة سيناريوهات</t>
+          <t>28 مبادرة على 4 ركائز استراتيجية، 14 مؤشر أداء، وتوقعات 12 شهراً بثلاثة سيناريوهات</t>
         </is>
       </c>
     </row>
@@ -4379,10 +4379,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>37.1</v>
+        <v>55.6</v>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -4395,10 +4395,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>70.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>89.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -4411,10 +4411,10 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>48.5</v>
+        <v>62.2</v>
       </c>
       <c r="B4" t="n">
-        <v>70.90000000000001</v>
+        <v>61.2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -4427,10 +4427,10 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>55.7</v>
+        <v>66.2</v>
       </c>
       <c r="B5" t="n">
-        <v>68.2</v>
+        <v>57.3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -4443,10 +4443,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>56.1</v>
+        <v>66.5</v>
       </c>
       <c r="B6" t="n">
-        <v>88.7</v>
+        <v>87.2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -4459,10 +4459,10 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>37.4</v>
+        <v>55.8</v>
       </c>
       <c r="B7" t="n">
-        <v>87.7</v>
+        <v>85.7</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -4475,10 +4475,10 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>47.7</v>
+        <v>61.7</v>
       </c>
       <c r="B8" t="n">
-        <v>72.8</v>
+        <v>64</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -4491,10 +4491,10 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>59.9</v>
+        <v>68.7</v>
       </c>
       <c r="B9" t="n">
-        <v>86.09999999999999</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -4507,10 +4507,10 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>54.7</v>
+        <v>65.7</v>
       </c>
       <c r="B10" t="n">
-        <v>68.2</v>
+        <v>57.2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -4523,10 +4523,10 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>76.09999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="B11" t="n">
-        <v>86.5</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -4539,10 +4539,10 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>58.3</v>
+        <v>67.7</v>
       </c>
       <c r="B12" t="n">
-        <v>81.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -4555,10 +4555,10 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="B13" t="n">
-        <v>78.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -4571,10 +4571,10 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>89.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="B14" t="n">
-        <v>51.6</v>
+        <v>30.5</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -4587,10 +4587,10 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>74.09999999999999</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="B15" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -4603,10 +4603,10 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>82.3</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="B16" t="n">
-        <v>38.5</v>
+        <v>16</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -4619,10 +4619,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>84.8</v>
+        <v>82</v>
       </c>
       <c r="B17" t="n">
-        <v>59.1</v>
+        <v>38.8</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -4635,10 +4635,10 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>86.90000000000001</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="B18" t="n">
-        <v>56.5</v>
+        <v>35.9</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -4651,10 +4651,10 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>82.5</v>
+        <v>78.5</v>
       </c>
       <c r="B19" t="n">
-        <v>52.7</v>
+        <v>31.8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -4667,10 +4667,10 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>68.59999999999999</v>
+        <v>56.9</v>
       </c>
       <c r="B20" t="n">
-        <v>47.4</v>
+        <v>25.9</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -4683,10 +4683,10 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>73.7</v>
+        <v>64.8</v>
       </c>
       <c r="B21" t="n">
-        <v>45.1</v>
+        <v>23.4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -4699,10 +4699,10 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>84.2</v>
+        <v>81</v>
       </c>
       <c r="B22" t="n">
-        <v>49.9</v>
+        <v>28.7</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -4715,10 +4715,10 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>86</v>
+        <v>83.7</v>
       </c>
       <c r="B23" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -4731,10 +4731,10 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>44.4</v>
+        <v>45.7</v>
       </c>
       <c r="B24" t="n">
-        <v>46.2</v>
+        <v>55.5</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -4747,10 +4747,10 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>58.1</v>
+        <v>53.9</v>
       </c>
       <c r="B25" t="n">
-        <v>49.1</v>
+        <v>57.4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -4763,10 +4763,10 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>46</v>
+        <v>46.6</v>
       </c>
       <c r="B26" t="n">
-        <v>38.6</v>
+        <v>50.4</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -4779,10 +4779,10 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>43.6</v>
+        <v>45.2</v>
       </c>
       <c r="B27" t="n">
-        <v>37</v>
+        <v>49.4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -4795,10 +4795,10 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>54.8</v>
+        <v>51.9</v>
       </c>
       <c r="B28" t="n">
-        <v>50.2</v>
+        <v>58.2</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -4811,10 +4811,10 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>55.3</v>
+        <v>52.2</v>
       </c>
       <c r="B29" t="n">
-        <v>38.8</v>
+        <v>50.6</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -4827,10 +4827,10 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>53.1</v>
+        <v>50.9</v>
       </c>
       <c r="B30" t="n">
-        <v>39.7</v>
+        <v>51.1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -4843,10 +4843,10 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>64.7</v>
+        <v>37.6</v>
       </c>
       <c r="B31" t="n">
-        <v>13.6</v>
+        <v>23.3</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -4859,10 +4859,10 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>42.3</v>
+        <v>28.3</v>
       </c>
       <c r="B32" t="n">
-        <v>17.8</v>
+        <v>30.8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -4875,10 +4875,10 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>71.09999999999999</v>
+        <v>40.3</v>
       </c>
       <c r="B33" t="n">
-        <v>16.1</v>
+        <v>27.7</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -4891,10 +4891,10 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>48.3</v>
+        <v>30.8</v>
       </c>
       <c r="B34" t="n">
-        <v>11.9</v>
+        <v>20.3</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -4907,10 +4907,10 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>72</v>
+        <v>40.7</v>
       </c>
       <c r="B35" t="n">
-        <v>14.7</v>
+        <v>25.3</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -4923,10 +4923,10 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>44.8</v>
+        <v>29.3</v>
       </c>
       <c r="B36" t="n">
-        <v>22.1</v>
+        <v>38.5</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -4939,10 +4939,10 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>14.7</v>
+        <v>13.3</v>
       </c>
       <c r="B37" t="n">
-        <v>38</v>
+        <v>57.6</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -4955,10 +4955,10 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>31.7</v>
+        <v>33.7</v>
       </c>
       <c r="B38" t="n">
-        <v>55.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -4971,10 +4971,10 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>14.9</v>
+        <v>13.4</v>
       </c>
       <c r="B39" t="n">
-        <v>54.6</v>
+        <v>69.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4987,10 +4987,10 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>27.6</v>
+        <v>28.7</v>
       </c>
       <c r="B40" t="n">
-        <v>45.2</v>
+        <v>62.8</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -5003,10 +5003,10 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>31.7</v>
+        <v>33.7</v>
       </c>
       <c r="B41" t="n">
-        <v>40.8</v>
+        <v>59.6</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -5115,12 +5115,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>التنظيمات واللوائح</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>تحديث لائحة اشتراطات سكن العمالة الجماعي</t>
+          <t>تحديث لائحة اشتراطات السكن الجماعي للأفراد</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5173,12 +5173,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>التنظيمات واللوائح</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>إطار تصنيف مقدمي خدمات الإسكان العمالي</t>
+          <t>إطار تصنيف مقدمي خدمات الإسكان الجماعي</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>التنظيمات واللوائح</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>التنظيمات واللوائح</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5347,53 +5347,53 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>التطوير العمراني</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>مخطط المناطق النموذجية لإسكان العمالة (المرحلة الأولى)</t>
+          <t>مصفوفة الصلاحيات والأدوار للجهات المشاركة</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>الإدارة العامة للتخطيط العمراني</t>
+          <t>إدارة التنظيمات البلدية</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>مكتملة</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>38000000</v>
+        <v>700000</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>اعتماد المخطط التفصيلي للموقع الجنوبي</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>إضافة 45,000 سرير مرخص جديد</t>
+          <t>وضوح المساءلة عبر 9 جهات</t>
         </is>
       </c>
     </row>
@@ -5405,21 +5405,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>التطوير العمراني</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>نقل التجمعات العشوائية من الأحياء السكنية</t>
+          <t>سياسة تبادل البيانات مع الجهات الوطنية</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>الإدارة العامة للتخطيط العمراني</t>
+          <t>إدارة التنظيمات البلدية</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -5428,20 +5428,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2024-11-01</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>22500000</v>
+        <v>1200000</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>حصر التجمعات المستهدفة في السلي والمنصورية</t>
+          <t>توقيع اتفاقية التكامل مع المنصة الوطنية</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>إخلاء 120 موقعاً غير نظامي</t>
+          <t>تحديث تلقائي لبيانات العمالة شهرياً</t>
         </is>
       </c>
     </row>
@@ -5463,21 +5463,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>التطوير العمراني</t>
+          <t>الأنظمة والتشريعات</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>تأهيل البنية التحتية للمدينة العمالية بالمصفاة</t>
+          <t>إطار قياس أثر المبادرات الاستراتيجية</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>الإدارة العامة للتخطيط العمراني</t>
+          <t>إدارة التنظيمات البلدية</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -5486,20 +5486,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2025-04-20</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-12-10</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>17300000</v>
+        <v>900000</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>استكمال شبكات الصرف للمرحلة الثانية</t>
+          <t>اعتماد منهجية القياس</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>رفع الطاقة الاستيعابية 18,000 سرير</t>
+          <t>ربط الإنفاق بالأثر لكل مبادرة</t>
         </is>
       </c>
     </row>
@@ -5521,12 +5521,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>التطوير العمراني</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>دراسة مواءمة استعمالات الأراضي مع الطلب</t>
+          <t>مخطط المناطق النموذجية للسكن الجماعي (المرحلة الأولى)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5535,39 +5535,39 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>مكتملة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1600000</v>
+        <v>38000000</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>اعتماد المخطط التفصيلي للموقع الجنوبي</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>خريطة فجوة معتمدة لتوجيه التراخيص</t>
+          <t>إضافة 45,000 سرير مرخص جديد</t>
         </is>
       </c>
     </row>
@@ -5579,53 +5579,53 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>الاستثمار والقطاع الخاص</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>طرح 6 فرص استثمارية لمجمعات سكن عمالة</t>
+          <t>نقل التجمعات العشوائية من الأحياء السكنية</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>إدارة الاستثمار والشراكات</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>متأخرة</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2025-05-01</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2027-02-28</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5400000</v>
+        <v>22500000</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>إغلاق التأهيل المسبق للمطورين</t>
+          <t>حصر التجمعات المستهدفة في السلي والمنصورية</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>مرتفع</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>استقطاب استثمارات بـ 1.2 مليار ريال</t>
+          <t>إخلاء 120 موقعاً غير نظامي</t>
         </is>
       </c>
     </row>
@@ -5637,21 +5637,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>الاستثمار والقطاع الخاص</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>برنامج حوافز التراخيص للمطورين</t>
+          <t>تأهيل البنية التحتية للمدينة العمالية بالمصفاة</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>إدارة الاستثمار والشراكات</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -5660,30 +5660,30 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2025-01-15</t>
+          <t>2025-04-20</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3100000</v>
+        <v>17300000</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>إطلاق حزمة الحوافز الثانية</t>
+          <t>استكمال شبكات الصرف للمرحلة الثانية</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>تسريع دخول 25,000 سرير للسوق</t>
+          <t>رفع الطاقة الاستيعابية 18,000 سرير</t>
         </is>
       </c>
     </row>
@@ -5695,53 +5695,53 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>الاستثمار والقطاع الخاص</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>شراكة تشغيل المجمعات الحكومية مع القطاع الخاص</t>
+          <t>دراسة مواءمة استعمالات الأراضي مع الطلب</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>إدارة الاستثمار والشراكات</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>22</v>
+        <v>100</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>متوقفة</t>
+          <t>مكتملة</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2025-03-01</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2025-08-31</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>8700000</v>
+        <v>1600000</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>إعادة طرح كراسة الشروط</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>مرتفع</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>رفع كفاءة التشغيل وخفض التكاليف 30٪</t>
+          <t>خريطة فجوة معتمدة لتوجيه التراخيص</t>
         </is>
       </c>
     </row>
@@ -5753,21 +5753,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>الاستثمار والقطاع الخاص</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>منصة مطابقة العرض والطلب للمنشآت الصغيرة</t>
+          <t>التوأم الرقمي لمواقع السكن الجماعي</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>إدارة الاستثمار والشراكات</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -5776,20 +5776,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>2025-05-15</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2300000</v>
+        <v>9800000</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>اكتمال النموذج الأولي للمنصة</t>
+          <t>مسح ثلاثي الأبعاد لأول 200 منشأة</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>خدمة 8,000 منشأة صغيرة ومتناهية الصغر</t>
+          <t>خفض زيارات التحقق الميدانية 35٪</t>
         </is>
       </c>
     </row>
@@ -5811,21 +5811,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>الرقابة والامتثال</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>برنامج الرقابة الوقائية بالنمذجة التنبؤية</t>
+          <t>مكتب إدارة بيانات السكن الجماعي</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>الإدارة العامة للرقابة الميدانية</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -5834,30 +5834,30 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2025-02-15</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-12-20</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>4800000</v>
+        <v>2900000</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>تشغيل نموذج المخاطر على بيانات 6 أشهر</t>
+          <t>إطلاق قاموس البيانات الموحد</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>رفع دقة استهداف الجولات إلى 75٪</t>
+          <t>مصدر واحد موثوق لكل مؤشرات القطاع</t>
         </is>
       </c>
     </row>
@@ -5869,21 +5869,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>الرقابة والامتثال</t>
+          <t>النموذج الحضري</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>حملة الامتثال الشامل بالقطاع الجنوبي</t>
+          <t>لوحات المؤشرات التنفيذية الموحدة</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>الإدارة العامة للرقابة الميدانية</t>
+          <t>الإدارة العامة للتخطيط العمراني</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -5892,20 +5892,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2025-09-01</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>3500000</v>
+        <v>1500000</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>تغطية آخر 60 موقعاً عالي الخطورة</t>
+          <t>ربط مصادر البيانات المتبقية</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>خفض المخالفات الجسيمة 40٪ في الجنوب</t>
+          <t>قرارات أسرع بمعلومة موحدة</t>
         </is>
       </c>
     </row>
@@ -5927,53 +5927,53 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>الرقابة والامتثال</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ربط أجهزة المفتشين بمنظومة بلدي الرقابية</t>
+          <t>طرح 6 فرص استثمارية لمجمعات السكن الجماعي</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>الإدارة العامة للرقابة الميدانية</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>مكتملة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2027-02-28</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2100000</v>
+        <v>5400000</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>إغلاق التأهيل المسبق للمطورين</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>أتمتة 100٪ من محاضر الضبط</t>
+          <t>استقطاب استثمارات بـ 1.2 مليار ريال</t>
         </is>
       </c>
     </row>
@@ -5985,53 +5985,53 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>الرقابة والامتثال</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>إطار التفتيش المشترك مع الدفاع المدني</t>
+          <t>برنامج حوافز التراخيص للمطورين</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>الإدارة العامة للرقابة الميدانية</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>متأخرة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2025-01-20</t>
+          <t>2025-01-15</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1400000</v>
+        <v>3100000</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>اعتماد بروتوكول الجولات المشتركة</t>
+          <t>إطلاق حزمة الحوافز الثانية</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>مرتفع</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>توحيد ضبط اشتراطات السلامة</t>
+          <t>تسريع دخول 25,000 سرير للسوق</t>
         </is>
       </c>
     </row>
@@ -6043,30 +6043,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>الحوكمة</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>مكتب إدارة بيانات سكن العمالة</t>
+          <t>شراكة تشغيل المجمعات الحكومية مع القطاع الخاص</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>مكتب الحوكمة والالتزام</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>متوقفة</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -6075,21 +6075,21 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2900000</v>
+        <v>8700000</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>إطلاق قاموس البيانات الموحد</t>
+          <t>إعادة طرح كراسة الشروط</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>مرتفع</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>مصدر واحد موثوق لكل مؤشرات القطاع</t>
+          <t>رفع كفاءة التشغيل وخفض التكاليف 30٪</t>
         </is>
       </c>
     </row>
@@ -6101,53 +6101,53 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>الحوكمة</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>مصفوفة الصلاحيات والأدوار للجهات المشاركة</t>
+          <t>منصة مطابقة العرض والطلب للمنشآت الصغيرة</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>مكتب الحوكمة والالتزام</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>47</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>مكتملة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2024-08-01</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>700000</v>
+        <v>2300000</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>اكتمال النموذج الأولي للمنصة</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>وضوح المساءلة عبر 9 جهات</t>
+          <t>خدمة 8,000 منشأة صغيرة ومتناهية الصغر</t>
         </is>
       </c>
     </row>
@@ -6159,53 +6159,53 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>الحوكمة</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>سياسة تبادل البيانات مع الجهات الوطنية</t>
+          <t>ملتقى الرياض السنوي للإسكان الجماعي</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>مكتب الحوكمة والالتزام</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>متأخرة</t>
+          <t>متوقفة</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2025-04-01</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1200000</v>
+        <v>3200000</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>توقيع اتفاقية التكامل مع المنصة الوطنية</t>
+          <t>تحديد موعد وشركاء النسخة الأولى</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>مرتفع</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>تحديث تلقائي لبيانات العمالة شهرياً</t>
+          <t>منصة سنوية للقطاعين العام والخاص</t>
         </is>
       </c>
     </row>
@@ -6217,21 +6217,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>الحوكمة</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>إطار قياس أثر المبادرات الاستراتيجية</t>
+          <t>حملة «سكن آمن» لتوعية أصحاب العمل</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>مكتب الحوكمة والالتزام</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -6240,30 +6240,30 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2025-07-01</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2026-12-20</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>900000</v>
+        <v>2400000</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>اعتماد منهجية القياس</t>
+          <t>إطلاق الموجة الثالثة من الحملة</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>ربط الإنفاق بالأثر لكل مبادرة</t>
+          <t>وصول 50,000 منشأة مستهدفة</t>
         </is>
       </c>
     </row>
@@ -6275,43 +6275,43 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>التحول الرقمي</t>
+          <t>الاستثمار والقطاع الخاص</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>منصة الترخيص الإلكتروني الموحد لسكن العمالة</t>
+          <t>دليل المستأجر العامل بست لغات</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>إدارة التحول الرقمي</t>
+          <t>إدارة الاستثمار والشراكات</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>مكتملة</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2024-12-01</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>12500000</v>
+        <v>600000</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>إطلاق خدمة رخص البناء رقمياً</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>إصدار 95٪ من الرخص إلكترونياً</t>
+          <t>تمكين العمال من معرفة حقوقهم السكنية</t>
         </is>
       </c>
     </row>
@@ -6333,21 +6333,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>التحول الرقمي</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>التوأم الرقمي لمواقع سكن العمالة</t>
+          <t>برنامج الرقابة الوقائية بالنمذجة التنبؤية</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>إدارة التحول الرقمي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -6356,20 +6356,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2025-05-15</t>
+          <t>2025-02-15</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2026-12-20</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>9800000</v>
+        <v>4800000</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>مسح ثلاثي الأبعاد لأول 200 منشأة</t>
+          <t>تشغيل نموذج المخاطر على بيانات 6 أشهر</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>خفض زيارات التحقق الميدانية 35٪</t>
+          <t>رفع دقة استهداف الجولات إلى 75٪</t>
         </is>
       </c>
     </row>
@@ -6391,43 +6391,43 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>التحول الرقمي</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>تطبيق البلاغات المجتمعية عن السكن العشوائي</t>
+          <t>حملة الامتثال الشامل بالقطاع الجنوبي</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>إدارة التحول الرقمي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>مكتملة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2025-01-01</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1800000</v>
+        <v>3500000</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>تغطية آخر 60 موقعاً عالي الخطورة</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>استقبال 1,500 بلاغ نوعي سنوياً</t>
+          <t>خفض المخالفات الجسيمة 40٪ في الجنوب</t>
         </is>
       </c>
     </row>
@@ -6449,43 +6449,43 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>التحول الرقمي</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>لوحات المؤشرات التنفيذية الموحدة</t>
+          <t>ربط أجهزة المفتشين بمنظومة بلدي الرقابية</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>إدارة التحول الرقمي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>مكتملة</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2025-06-01</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1500000</v>
+        <v>2100000</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>ربط مصادر البيانات المتبقية</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>قرارات أسرع بمعلومة موحدة</t>
+          <t>أتمتة 100٪ من محاضر الضبط</t>
         </is>
       </c>
     </row>
@@ -6507,53 +6507,53 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>التواصل والتوعية</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>حملة «سكن آمن» لتوعية أصحاب العمل</t>
+          <t>إطار التفتيش المشترك مع الدفاع المدني</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>إدارة التواصل المؤسسي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>متأخرة</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2025-04-01</t>
+          <t>2025-01-20</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-12-20</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>2400000</v>
+        <v>1400000</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>إطلاق الموجة الثالثة من الحملة</t>
+          <t>اعتماد بروتوكول الجولات المشتركة</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>منخفض</t>
+          <t>مرتفع</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>وصول 50,000 منشأة مستهدفة</t>
+          <t>توحيد ضبط اشتراطات السلامة</t>
         </is>
       </c>
     </row>
@@ -6565,43 +6565,43 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>التواصل والتوعية</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>دليل المستأجر العامل بست لغات</t>
+          <t>منصة الترخيص الإلكتروني الموحد للسكن الجماعي</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>إدارة التواصل المؤسسي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>مكتملة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>600000</v>
+        <v>12500000</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>إطلاق خدمة رخص البناء رقمياً</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>تمكين العمال من معرفة حقوقهم السكنية</t>
+          <t>إصدار 95٪ من الرخص إلكترونياً</t>
         </is>
       </c>
     </row>
@@ -6623,53 +6623,53 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>التواصل والتوعية</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>برنامج سفراء الامتثال في المنشآت الكبرى</t>
+          <t>تطبيق البلاغات المجتمعية عن السكن العشوائي</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>إدارة التواصل المؤسسي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>في المسار</t>
+          <t>مكتملة</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1100000</v>
+        <v>1800000</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>تدريب الدفعة الثانية (120 سفيراً)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>قناة امتثال ذاتي داخل أكبر 500 منشأة</t>
+          <t>استقبال 1,500 بلاغ نوعي سنوياً</t>
         </is>
       </c>
     </row>
@@ -6681,43 +6681,43 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>التواصل والتوعية</t>
+          <t>الرقابة</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ملتقى الرياض السنوي لإسكان العمالة</t>
+          <t>برنامج سفراء الامتثال في المنشآت الكبرى</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>إدارة التواصل المؤسسي</t>
+          <t>الإدارة العامة للرقابة الميدانية</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>متوقفة</t>
+          <t>في المسار</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2025-06-01</t>
+          <t>2025-09-15</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>3200000</v>
+        <v>1100000</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>تحديد موعد وشركاء النسخة الأولى</t>
+          <t>تدريب الدفعة الثانية (120 سفيراً)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -6727,7 +6727,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>منصة سنوية للقطاعين العام والخاص</t>
+          <t>قناة امتثال ذاتي داخل أكبر 500 منشأة</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7900,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ثلاث مبادرات تقترب من الإغلاق خلال 90 يوماً: منصة الترخيص الإلكتروني الموحد لسكن العمالة (91٪)، حملة الامتثال الشامل بالقطاع الجنوبي (86٪)، لوحات المؤشرات التنفيذية الموحدة (84٪).</t>
+          <t>ثلاث مبادرات تقترب من الإغلاق خلال 90 يوماً: منصة الترخيص الإلكتروني الموحد للسكن الجماعي (91٪)، حملة الامتثال الشامل بالقطاع الجنوبي (86٪)، لوحات المؤشرات التنفيذية الموحدة (84٪).</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9438,10 +9438,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9466,10 +9466,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9494,10 +9494,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9525,7 +9525,7 @@
         <v>21</v>
       </c>
       <c r="E5" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -9550,10 +9550,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E6" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -11464,10 +11464,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>69.3</v>
+        <v>39.5</v>
       </c>
       <c r="G2" t="n">
-        <v>21.1</v>
+        <v>36.7</v>
       </c>
       <c r="H2" t="n">
         <v>17388</v>
@@ -11529,10 +11529,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>36.1</v>
+        <v>25.7</v>
       </c>
       <c r="G3" t="n">
-        <v>12.2</v>
+        <v>20.7</v>
       </c>
       <c r="H3" t="n">
         <v>8649</v>
@@ -11594,10 +11594,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>72.59999999999999</v>
+        <v>40.9</v>
       </c>
       <c r="G4" t="n">
-        <v>13.7</v>
+        <v>23.5</v>
       </c>
       <c r="H4" t="n">
         <v>11364</v>
@@ -11659,10 +11659,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>43.7</v>
+        <v>28.9</v>
       </c>
       <c r="G5" t="n">
-        <v>22.7</v>
+        <v>39.7</v>
       </c>
       <c r="H5" t="n">
         <v>11849</v>
@@ -11724,10 +11724,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>28.6</v>
+        <v>22.6</v>
       </c>
       <c r="G6" t="n">
-        <v>11.1</v>
+        <v>18.8</v>
       </c>
       <c r="H6" t="n">
         <v>17264</v>
@@ -11789,10 +11789,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>52.3</v>
+        <v>32.5</v>
       </c>
       <c r="G7" t="n">
-        <v>20.2</v>
+        <v>35.2</v>
       </c>
       <c r="H7" t="n">
         <v>16442</v>
@@ -11854,10 +11854,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>73.90000000000001</v>
+        <v>41.4</v>
       </c>
       <c r="G8" t="n">
-        <v>15</v>
+        <v>25.8</v>
       </c>
       <c r="H8" t="n">
         <v>20045</v>
@@ -11919,10 +11919,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>79.8</v>
+        <v>43.9</v>
       </c>
       <c r="G9" t="n">
-        <v>11.1</v>
+        <v>18.7</v>
       </c>
       <c r="H9" t="n">
         <v>8999</v>
@@ -11984,10 +11984,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>45.4</v>
+        <v>29.6</v>
       </c>
       <c r="G10" t="n">
-        <v>12.2</v>
+        <v>20.7</v>
       </c>
       <c r="H10" t="n">
         <v>836</v>
@@ -12049,10 +12049,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>65.3</v>
+        <v>37.9</v>
       </c>
       <c r="G11" t="n">
-        <v>19.3</v>
+        <v>33.6</v>
       </c>
       <c r="H11" t="n">
         <v>995</v>
@@ -12114,10 +12114,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>43.9</v>
+        <v>29</v>
       </c>
       <c r="G12" t="n">
-        <v>19.1</v>
+        <v>33.1</v>
       </c>
       <c r="H12" t="n">
         <v>1105</v>
@@ -12179,10 +12179,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>46.3</v>
+        <v>30</v>
       </c>
       <c r="G13" t="n">
-        <v>16.8</v>
+        <v>29</v>
       </c>
       <c r="H13" t="n">
         <v>583</v>
@@ -12244,10 +12244,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>34.9</v>
+        <v>25.2</v>
       </c>
       <c r="G14" t="n">
-        <v>10</v>
+        <v>16.7</v>
       </c>
       <c r="H14" t="n">
         <v>540</v>
@@ -12309,10 +12309,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>55.3</v>
+        <v>33.7</v>
       </c>
       <c r="G15" t="n">
-        <v>12.5</v>
+        <v>21.2</v>
       </c>
       <c r="H15" t="n">
         <v>971</v>
@@ -12374,10 +12374,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>20.4</v>
+        <v>19.2</v>
       </c>
       <c r="G16" t="n">
-        <v>19.6</v>
+        <v>34.1</v>
       </c>
       <c r="H16" t="n">
         <v>917</v>
@@ -12439,10 +12439,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.7</v>
+        <v>24.7</v>
       </c>
       <c r="G17" t="n">
-        <v>22.6</v>
+        <v>39.4</v>
       </c>
       <c r="H17" t="n">
         <v>751</v>
@@ -12504,10 +12504,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>24.3</v>
+        <v>20.8</v>
       </c>
       <c r="G18" t="n">
-        <v>12.6</v>
+        <v>21.4</v>
       </c>
       <c r="H18" t="n">
         <v>877</v>
@@ -12569,10 +12569,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>32.9</v>
+        <v>24.4</v>
       </c>
       <c r="G19" t="n">
-        <v>11</v>
+        <v>18.6</v>
       </c>
       <c r="H19" t="n">
         <v>825</v>
@@ -12634,10 +12634,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>54.6</v>
+        <v>33.4</v>
       </c>
       <c r="G20" t="n">
-        <v>12.6</v>
+        <v>21.6</v>
       </c>
       <c r="H20" t="n">
         <v>605</v>
@@ -12699,10 +12699,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>68.40000000000001</v>
+        <v>39.2</v>
       </c>
       <c r="G21" t="n">
-        <v>11.9</v>
+        <v>20.1</v>
       </c>
       <c r="H21" t="n">
         <v>876</v>
@@ -12764,10 +12764,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>59.5</v>
+        <v>35.5</v>
       </c>
       <c r="G22" t="n">
-        <v>14.3</v>
+        <v>24.6</v>
       </c>
       <c r="H22" t="n">
         <v>1136</v>
@@ -12829,10 +12829,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>48</v>
+        <v>30.7</v>
       </c>
       <c r="G23" t="n">
-        <v>19.9</v>
+        <v>34.7</v>
       </c>
       <c r="H23" t="n">
         <v>983</v>
@@ -12894,10 +12894,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>34.3</v>
+        <v>25</v>
       </c>
       <c r="G24" t="n">
-        <v>14.9</v>
+        <v>25.7</v>
       </c>
       <c r="H24" t="n">
         <v>600</v>
@@ -12959,10 +12959,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>47.4</v>
+        <v>30.4</v>
       </c>
       <c r="G25" t="n">
-        <v>22.9</v>
+        <v>40.1</v>
       </c>
       <c r="H25" t="n">
         <v>600</v>
@@ -13024,10 +13024,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>20.6</v>
+        <v>19.2</v>
       </c>
       <c r="G26" t="n">
-        <v>18.3</v>
+        <v>31.8</v>
       </c>
       <c r="H26" t="n">
         <v>384</v>
@@ -13089,10 +13089,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>79.8</v>
+        <v>43.9</v>
       </c>
       <c r="G27" t="n">
-        <v>10.1</v>
+        <v>17</v>
       </c>
       <c r="H27" t="n">
         <v>489</v>
@@ -13154,10 +13154,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>50.4</v>
+        <v>31.6</v>
       </c>
       <c r="G28" t="n">
-        <v>11</v>
+        <v>18.6</v>
       </c>
       <c r="H28" t="n">
         <v>454</v>
@@ -13219,10 +13219,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>72.90000000000001</v>
+        <v>41</v>
       </c>
       <c r="G29" t="n">
-        <v>22.2</v>
+        <v>38.7</v>
       </c>
       <c r="H29" t="n">
         <v>600</v>
@@ -13284,10 +13284,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>37.1</v>
+        <v>26.1</v>
       </c>
       <c r="G30" t="n">
-        <v>15.6</v>
+        <v>26.8</v>
       </c>
       <c r="H30" t="n">
         <v>434</v>
@@ -13349,10 +13349,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>62.2</v>
+        <v>36.6</v>
       </c>
       <c r="G31" t="n">
-        <v>18.2</v>
+        <v>31.5</v>
       </c>
       <c r="H31" t="n">
         <v>439</v>
@@ -13414,10 +13414,10 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>75.3</v>
+        <v>67.3</v>
       </c>
       <c r="G32" t="n">
-        <v>33.8</v>
+        <v>10.9</v>
       </c>
       <c r="H32" t="n">
         <v>22000</v>
@@ -13479,10 +13479,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>71.90000000000001</v>
+        <v>62.1</v>
       </c>
       <c r="G33" t="n">
-        <v>60.9</v>
+        <v>40.8</v>
       </c>
       <c r="H33" t="n">
         <v>17965</v>
@@ -13544,10 +13544,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>68.8</v>
+        <v>57.3</v>
       </c>
       <c r="G34" t="n">
-        <v>50.3</v>
+        <v>29.1</v>
       </c>
       <c r="H34" t="n">
         <v>9303</v>
@@ -13609,10 +13609,10 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>84</v>
+        <v>80.8</v>
       </c>
       <c r="G35" t="n">
-        <v>42.1</v>
+        <v>20</v>
       </c>
       <c r="H35" t="n">
         <v>20542</v>
@@ -13674,10 +13674,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>89.7</v>
+        <v>89.5</v>
       </c>
       <c r="G36" t="n">
-        <v>36.4</v>
+        <v>13.7</v>
       </c>
       <c r="H36" t="n">
         <v>13954</v>
@@ -13739,10 +13739,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>72.2</v>
+        <v>62.5</v>
       </c>
       <c r="G37" t="n">
-        <v>34.3</v>
+        <v>11.4</v>
       </c>
       <c r="H37" t="n">
         <v>18272</v>
@@ -13804,10 +13804,10 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>68</v>
+        <v>56.1</v>
       </c>
       <c r="G38" t="n">
-        <v>59.8</v>
+        <v>39.6</v>
       </c>
       <c r="H38" t="n">
         <v>21949</v>
@@ -13869,10 +13869,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>83.09999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>60.3</v>
+        <v>40.1</v>
       </c>
       <c r="H39" t="n">
         <v>10675</v>
@@ -13934,10 +13934,10 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>76</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G40" t="n">
-        <v>35</v>
+        <v>12.2</v>
       </c>
       <c r="H40" t="n">
         <v>10947</v>
@@ -13999,10 +13999,10 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>81.7</v>
+        <v>77.2</v>
       </c>
       <c r="G41" t="n">
-        <v>52.2</v>
+        <v>31.2</v>
       </c>
       <c r="H41" t="n">
         <v>10393</v>
@@ -14064,10 +14064,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>85.09999999999999</v>
+        <v>82.5</v>
       </c>
       <c r="G42" t="n">
-        <v>39.3</v>
+        <v>17</v>
       </c>
       <c r="H42" t="n">
         <v>511</v>
@@ -14129,10 +14129,10 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>78.2</v>
+        <v>71.8</v>
       </c>
       <c r="G43" t="n">
-        <v>49.2</v>
+        <v>27.8</v>
       </c>
       <c r="H43" t="n">
         <v>1053</v>
@@ -14194,10 +14194,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>78</v>
+        <v>71.5</v>
       </c>
       <c r="G44" t="n">
-        <v>56.2</v>
+        <v>35.6</v>
       </c>
       <c r="H44" t="n">
         <v>777</v>
@@ -14259,10 +14259,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>89.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G45" t="n">
-        <v>50.3</v>
+        <v>29.1</v>
       </c>
       <c r="H45" t="n">
         <v>891</v>
@@ -14324,10 +14324,10 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>81.5</v>
+        <v>76.8</v>
       </c>
       <c r="G46" t="n">
-        <v>53.9</v>
+        <v>33</v>
       </c>
       <c r="H46" t="n">
         <v>652</v>
@@ -14389,10 +14389,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>77.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="G47" t="n">
-        <v>59.3</v>
+        <v>39</v>
       </c>
       <c r="H47" t="n">
         <v>912</v>
@@ -14454,10 +14454,10 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>87.7</v>
+        <v>86.5</v>
       </c>
       <c r="G48" t="n">
-        <v>54.6</v>
+        <v>33.8</v>
       </c>
       <c r="H48" t="n">
         <v>808</v>
@@ -14519,10 +14519,10 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>77.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="G49" t="n">
-        <v>54.8</v>
+        <v>34.1</v>
       </c>
       <c r="H49" t="n">
         <v>556</v>
@@ -14584,10 +14584,10 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>84.8</v>
+        <v>82</v>
       </c>
       <c r="G50" t="n">
-        <v>48.1</v>
+        <v>26.7</v>
       </c>
       <c r="H50" t="n">
         <v>890</v>
@@ -14649,10 +14649,10 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>74</v>
+        <v>65.3</v>
       </c>
       <c r="G51" t="n">
-        <v>35.2</v>
+        <v>12.5</v>
       </c>
       <c r="H51" t="n">
         <v>689</v>
@@ -14714,10 +14714,10 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>73.2</v>
+        <v>64</v>
       </c>
       <c r="G52" t="n">
-        <v>42.7</v>
+        <v>20.7</v>
       </c>
       <c r="H52" t="n">
         <v>946</v>
@@ -14779,10 +14779,10 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>69.8</v>
+        <v>58.7</v>
       </c>
       <c r="G53" t="n">
-        <v>37.4</v>
+        <v>14.8</v>
       </c>
       <c r="H53" t="n">
         <v>548</v>
@@ -14844,10 +14844,10 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>83.3</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G54" t="n">
-        <v>53.5</v>
+        <v>32.6</v>
       </c>
       <c r="H54" t="n">
         <v>821</v>
@@ -14909,10 +14909,10 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>77.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G55" t="n">
-        <v>42.6</v>
+        <v>20.6</v>
       </c>
       <c r="H55" t="n">
         <v>707</v>
@@ -14974,10 +14974,10 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>77.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>39</v>
+        <v>16.6</v>
       </c>
       <c r="H56" t="n">
         <v>1004</v>
@@ -15039,10 +15039,10 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>76.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="G57" t="n">
-        <v>55.3</v>
+        <v>34.6</v>
       </c>
       <c r="H57" t="n">
         <v>635</v>
@@ -15104,10 +15104,10 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>78.3</v>
+        <v>72</v>
       </c>
       <c r="G58" t="n">
-        <v>54.7</v>
+        <v>34</v>
       </c>
       <c r="H58" t="n">
         <v>600</v>
@@ -15172,7 +15172,7 @@
         <v>90</v>
       </c>
       <c r="G59" t="n">
-        <v>43.1</v>
+        <v>21.2</v>
       </c>
       <c r="H59" t="n">
         <v>285</v>
@@ -15234,10 +15234,10 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>85.2</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G60" t="n">
-        <v>51.9</v>
+        <v>30.9</v>
       </c>
       <c r="H60" t="n">
         <v>600</v>
@@ -15299,10 +15299,10 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>88.90000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="G61" t="n">
-        <v>38.8</v>
+        <v>16.4</v>
       </c>
       <c r="H61" t="n">
         <v>540</v>
@@ -15364,10 +15364,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>81.7</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="G62" t="n">
-        <v>39.9</v>
+        <v>17.6</v>
       </c>
       <c r="H62" t="n">
         <v>495</v>
@@ -15429,10 +15429,10 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>82.7</v>
+        <v>78.8</v>
       </c>
       <c r="G63" t="n">
-        <v>49.4</v>
+        <v>28</v>
       </c>
       <c r="H63" t="n">
         <v>600</v>
@@ -15494,10 +15494,10 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>78.2</v>
+        <v>71.8</v>
       </c>
       <c r="G64" t="n">
-        <v>40.4</v>
+        <v>18.2</v>
       </c>
       <c r="H64" t="n">
         <v>422</v>
@@ -15559,10 +15559,10 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>71.7</v>
+        <v>61.7</v>
       </c>
       <c r="G65" t="n">
-        <v>50.6</v>
+        <v>29.4</v>
       </c>
       <c r="H65" t="n">
         <v>458</v>
@@ -15624,10 +15624,10 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>52.3</v>
+        <v>50.4</v>
       </c>
       <c r="G66" t="n">
-        <v>54.3</v>
+        <v>60.9</v>
       </c>
       <c r="H66" t="n">
         <v>17472</v>
@@ -15689,10 +15689,10 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>49.3</v>
+        <v>48.6</v>
       </c>
       <c r="G67" t="n">
-        <v>52.3</v>
+        <v>59.6</v>
       </c>
       <c r="H67" t="n">
         <v>9427</v>
@@ -15754,10 +15754,10 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>45.4</v>
+        <v>46.2</v>
       </c>
       <c r="G68" t="n">
-        <v>52.9</v>
+        <v>59.9</v>
       </c>
       <c r="H68" t="n">
         <v>18674</v>
@@ -15819,10 +15819,10 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>45.6</v>
+        <v>46.3</v>
       </c>
       <c r="G69" t="n">
-        <v>44.5</v>
+        <v>54.3</v>
       </c>
       <c r="H69" t="n">
         <v>20505</v>
@@ -15884,10 +15884,10 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>51.4</v>
+        <v>49.8</v>
       </c>
       <c r="G70" t="n">
-        <v>49</v>
+        <v>57.4</v>
       </c>
       <c r="H70" t="n">
         <v>9680</v>
@@ -15949,10 +15949,10 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>40.6</v>
+        <v>43.3</v>
       </c>
       <c r="G71" t="n">
-        <v>52.9</v>
+        <v>59.9</v>
       </c>
       <c r="H71" t="n">
         <v>8842</v>
@@ -16014,10 +16014,10 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>59</v>
+        <v>54.4</v>
       </c>
       <c r="G72" t="n">
-        <v>49.5</v>
+        <v>57.7</v>
       </c>
       <c r="H72" t="n">
         <v>497</v>
@@ -16079,10 +16079,10 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>44.3</v>
+        <v>45.6</v>
       </c>
       <c r="G73" t="n">
-        <v>45.2</v>
+        <v>54.8</v>
       </c>
       <c r="H73" t="n">
         <v>517</v>
@@ -16144,10 +16144,10 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>59.5</v>
+        <v>54.7</v>
       </c>
       <c r="G74" t="n">
-        <v>46</v>
+        <v>55.3</v>
       </c>
       <c r="H74" t="n">
         <v>878</v>
@@ -16209,10 +16209,10 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>59.6</v>
+        <v>54.8</v>
       </c>
       <c r="G75" t="n">
-        <v>52.5</v>
+        <v>59.7</v>
       </c>
       <c r="H75" t="n">
         <v>599</v>
@@ -16274,10 +16274,10 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>44.5</v>
+        <v>45.7</v>
       </c>
       <c r="G76" t="n">
-        <v>38.8</v>
+        <v>50.5</v>
       </c>
       <c r="H76" t="n">
         <v>935</v>
@@ -16339,10 +16339,10 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>54.2</v>
+        <v>51.5</v>
       </c>
       <c r="G77" t="n">
-        <v>37.7</v>
+        <v>49.8</v>
       </c>
       <c r="H77" t="n">
         <v>823</v>
@@ -16404,10 +16404,10 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>59.5</v>
+        <v>54.7</v>
       </c>
       <c r="G78" t="n">
-        <v>46.6</v>
+        <v>55.7</v>
       </c>
       <c r="H78" t="n">
         <v>556</v>
@@ -16469,10 +16469,10 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>52.8</v>
+        <v>50.7</v>
       </c>
       <c r="G79" t="n">
-        <v>50.8</v>
+        <v>58.5</v>
       </c>
       <c r="H79" t="n">
         <v>399</v>
@@ -16534,10 +16534,10 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>57.5</v>
+        <v>53.5</v>
       </c>
       <c r="G80" t="n">
-        <v>47.1</v>
+        <v>56</v>
       </c>
       <c r="H80" t="n">
         <v>974</v>
@@ -16599,10 +16599,10 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>49.6</v>
+        <v>48.7</v>
       </c>
       <c r="G81" t="n">
-        <v>42.2</v>
+        <v>52.8</v>
       </c>
       <c r="H81" t="n">
         <v>435</v>
@@ -16664,10 +16664,10 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G82" t="n">
-        <v>53.1</v>
+        <v>60.1</v>
       </c>
       <c r="H82" t="n">
         <v>834</v>
@@ -16729,10 +16729,10 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>56.4</v>
+        <v>52.9</v>
       </c>
       <c r="G83" t="n">
-        <v>43.4</v>
+        <v>53.6</v>
       </c>
       <c r="H83" t="n">
         <v>697</v>
@@ -16794,10 +16794,10 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>51.5</v>
+        <v>49.9</v>
       </c>
       <c r="G84" t="n">
-        <v>49.4</v>
+        <v>57.6</v>
       </c>
       <c r="H84" t="n">
         <v>856</v>
@@ -16859,10 +16859,10 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>43.1</v>
+        <v>44.9</v>
       </c>
       <c r="G85" t="n">
-        <v>38.7</v>
+        <v>50.4</v>
       </c>
       <c r="H85" t="n">
         <v>237</v>
@@ -16924,10 +16924,10 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>43.1</v>
+        <v>44.9</v>
       </c>
       <c r="G86" t="n">
-        <v>43.6</v>
+        <v>53.7</v>
       </c>
       <c r="H86" t="n">
         <v>449</v>
@@ -16989,10 +16989,10 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>49.4</v>
+        <v>48.6</v>
       </c>
       <c r="G87" t="n">
-        <v>35.7</v>
+        <v>48.5</v>
       </c>
       <c r="H87" t="n">
         <v>487</v>
@@ -17054,10 +17054,10 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>54.1</v>
+        <v>51.5</v>
       </c>
       <c r="G88" t="n">
-        <v>49.8</v>
+        <v>57.8</v>
       </c>
       <c r="H88" t="n">
         <v>229</v>
@@ -17119,10 +17119,10 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>41.4</v>
+        <v>43.9</v>
       </c>
       <c r="G89" t="n">
-        <v>39.9</v>
+        <v>51.3</v>
       </c>
       <c r="H89" t="n">
         <v>297</v>
@@ -17184,10 +17184,10 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>55.8</v>
+        <v>52.5</v>
       </c>
       <c r="G90" t="n">
-        <v>48.1</v>
+        <v>56.8</v>
       </c>
       <c r="H90" t="n">
         <v>364</v>
@@ -17249,10 +17249,10 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>48.5</v>
+        <v>48.1</v>
       </c>
       <c r="G91" t="n">
-        <v>46.4</v>
+        <v>55.6</v>
       </c>
       <c r="H91" t="n">
         <v>337</v>
@@ -17314,10 +17314,10 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>25</v>
+        <v>25.6</v>
       </c>
       <c r="G92" t="n">
-        <v>55.9</v>
+        <v>70.5</v>
       </c>
       <c r="H92" t="n">
         <v>14892</v>
@@ -17379,10 +17379,10 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>31.9</v>
+        <v>33.9</v>
       </c>
       <c r="G93" t="n">
-        <v>43.9</v>
+        <v>61.8</v>
       </c>
       <c r="H93" t="n">
         <v>17872</v>
@@ -17444,10 +17444,10 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>31.4</v>
+        <v>33.3</v>
       </c>
       <c r="G94" t="n">
-        <v>44.8</v>
+        <v>62.5</v>
       </c>
       <c r="H94" t="n">
         <v>17077</v>
@@ -17509,10 +17509,10 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>18.7</v>
+        <v>18</v>
       </c>
       <c r="G95" t="n">
-        <v>49.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="H95" t="n">
         <v>8222</v>
@@ -17574,10 +17574,10 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>18.6</v>
+        <v>17.9</v>
       </c>
       <c r="G96" t="n">
-        <v>50.3</v>
+        <v>66.5</v>
       </c>
       <c r="H96" t="n">
         <v>9305</v>
@@ -17639,10 +17639,10 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>25.3</v>
+        <v>25.9</v>
       </c>
       <c r="G97" t="n">
-        <v>43</v>
+        <v>61.2</v>
       </c>
       <c r="H97" t="n">
         <v>11032</v>
@@ -17704,10 +17704,10 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>27.5</v>
+        <v>28.5</v>
       </c>
       <c r="G98" t="n">
-        <v>54.4</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="H98" t="n">
         <v>944</v>
@@ -17769,10 +17769,10 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>30.7</v>
+        <v>32.4</v>
       </c>
       <c r="G99" t="n">
-        <v>45.7</v>
+        <v>63.1</v>
       </c>
       <c r="H99" t="n">
         <v>436</v>
@@ -17834,10 +17834,10 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>17.7</v>
+        <v>16.8</v>
       </c>
       <c r="G100" t="n">
-        <v>40.5</v>
+        <v>59.4</v>
       </c>
       <c r="H100" t="n">
         <v>473</v>
@@ -17899,10 +17899,10 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>23.6</v>
+        <v>23.9</v>
       </c>
       <c r="G101" t="n">
-        <v>49.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H101" t="n">
         <v>608</v>
@@ -17964,10 +17964,10 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
       <c r="G102" t="n">
-        <v>45.1</v>
+        <v>62.7</v>
       </c>
       <c r="H102" t="n">
         <v>499</v>
@@ -18029,10 +18029,10 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="G103" t="n">
-        <v>46.6</v>
+        <v>63.8</v>
       </c>
       <c r="H103" t="n">
         <v>926</v>
@@ -18094,10 +18094,10 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>30.7</v>
+        <v>32.4</v>
       </c>
       <c r="G104" t="n">
-        <v>54.7</v>
+        <v>69.7</v>
       </c>
       <c r="H104" t="n">
         <v>970</v>
@@ -18159,10 +18159,10 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>23.4</v>
+        <v>23.7</v>
       </c>
       <c r="G105" t="n">
-        <v>38.8</v>
+        <v>58.2</v>
       </c>
       <c r="H105" t="n">
         <v>989</v>
@@ -18224,10 +18224,10 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>12.9</v>
+        <v>11</v>
       </c>
       <c r="G106" t="n">
-        <v>51.6</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="H106" t="n">
         <v>440</v>
@@ -18289,10 +18289,10 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>19.7</v>
+        <v>19.3</v>
       </c>
       <c r="G107" t="n">
-        <v>49.6</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H107" t="n">
         <v>992</v>
@@ -18357,7 +18357,7 @@
         <v>21.9</v>
       </c>
       <c r="G108" t="n">
-        <v>33.9</v>
+        <v>54.7</v>
       </c>
       <c r="H108" t="n">
         <v>723</v>
@@ -18419,10 +18419,10 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>26.9</v>
+        <v>27.9</v>
       </c>
       <c r="G109" t="n">
-        <v>43.8</v>
+        <v>61.8</v>
       </c>
       <c r="H109" t="n">
         <v>276</v>
@@ -18484,10 +18484,10 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>27.2</v>
+        <v>28.2</v>
       </c>
       <c r="G110" t="n">
-        <v>50.6</v>
+        <v>66.7</v>
       </c>
       <c r="H110" t="n">
         <v>307</v>
@@ -18549,10 +18549,10 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>20.9</v>
+        <v>20.6</v>
       </c>
       <c r="G111" t="n">
-        <v>50.4</v>
+        <v>66.5</v>
       </c>
       <c r="H111" t="n">
         <v>409</v>
@@ -18614,10 +18614,10 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>12.9</v>
+        <v>11.1</v>
       </c>
       <c r="G112" t="n">
-        <v>52.9</v>
+        <v>68.3</v>
       </c>
       <c r="H112" t="n">
         <v>358</v>
@@ -18679,10 +18679,10 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>19.2</v>
+        <v>18.6</v>
       </c>
       <c r="G113" t="n">
-        <v>43.8</v>
+        <v>61.8</v>
       </c>
       <c r="H113" t="n">
         <v>250</v>
@@ -18744,10 +18744,10 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>29.9</v>
+        <v>51.5</v>
       </c>
       <c r="G114" t="n">
-        <v>89.3</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H114" t="n">
         <v>11587</v>
@@ -18809,10 +18809,10 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>76.2</v>
+        <v>78</v>
       </c>
       <c r="G115" t="n">
-        <v>85.7</v>
+        <v>82.7</v>
       </c>
       <c r="H115" t="n">
         <v>13603</v>
@@ -18874,10 +18874,10 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>27.1</v>
+        <v>49.9</v>
       </c>
       <c r="G116" t="n">
-        <v>76.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="H116" t="n">
         <v>17992</v>
@@ -18939,10 +18939,10 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>52</v>
+        <v>64.2</v>
       </c>
       <c r="G117" t="n">
-        <v>78</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="H117" t="n">
         <v>11229</v>
@@ -19004,10 +19004,10 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>54.7</v>
+        <v>65.7</v>
       </c>
       <c r="G118" t="n">
-        <v>86.09999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H118" t="n">
         <v>12071</v>
@@ -19069,10 +19069,10 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>28.1</v>
+        <v>51.3</v>
       </c>
       <c r="G119" t="n">
-        <v>73.09999999999999</v>
+        <v>65</v>
       </c>
       <c r="H119" t="n">
         <v>16104</v>
@@ -19134,10 +19134,10 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>56.7</v>
+        <v>66.8</v>
       </c>
       <c r="G120" t="n">
-        <v>88.7</v>
+        <v>87.2</v>
       </c>
       <c r="H120" t="n">
         <v>13195</v>
@@ -19199,10 +19199,10 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>73.3</v>
+        <v>76.3</v>
       </c>
       <c r="G121" t="n">
-        <v>72.90000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H121" t="n">
         <v>19819</v>
@@ -19264,10 +19264,10 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>34.1</v>
+        <v>53.9</v>
       </c>
       <c r="G122" t="n">
-        <v>87.09999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="H122" t="n">
         <v>451</v>
@@ -19329,10 +19329,10 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>65.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="G123" t="n">
-        <v>85.40000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="H123" t="n">
         <v>955</v>
@@ -19394,10 +19394,10 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>22.2</v>
+        <v>47.1</v>
       </c>
       <c r="G124" t="n">
-        <v>86.90000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="H124" t="n">
         <v>1008</v>
@@ -19459,10 +19459,10 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>77.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G125" t="n">
-        <v>79.90000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="H125" t="n">
         <v>611</v>
@@ -19524,10 +19524,10 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>28.2</v>
+        <v>50.5</v>
       </c>
       <c r="G126" t="n">
-        <v>87.09999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="H126" t="n">
         <v>675</v>
@@ -19589,10 +19589,10 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>22.8</v>
+        <v>47.5</v>
       </c>
       <c r="G127" t="n">
-        <v>85.40000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="H127" t="n">
         <v>504</v>
@@ -19654,10 +19654,10 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>55</v>
+        <v>65.8</v>
       </c>
       <c r="G128" t="n">
-        <v>68.3</v>
+        <v>57.5</v>
       </c>
       <c r="H128" t="n">
         <v>1051</v>
@@ -19719,10 +19719,10 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>24.9</v>
+        <v>48.7</v>
       </c>
       <c r="G129" t="n">
-        <v>84.3</v>
+        <v>80.7</v>
       </c>
       <c r="H129" t="n">
         <v>616</v>
@@ -19784,10 +19784,10 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>28.4</v>
+        <v>54</v>
       </c>
       <c r="G130" t="n">
-        <v>69.40000000000001</v>
+        <v>62.9</v>
       </c>
       <c r="H130" t="n">
         <v>741</v>
@@ -19849,10 +19849,10 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>65.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G131" t="n">
-        <v>79.3</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="H131" t="n">
         <v>484</v>
@@ -19914,10 +19914,10 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>47.3</v>
+        <v>61.5</v>
       </c>
       <c r="G132" t="n">
-        <v>72.90000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H132" t="n">
         <v>999</v>
@@ -19979,10 +19979,10 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>24.4</v>
+        <v>48.4</v>
       </c>
       <c r="G133" t="n">
-        <v>85.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H133" t="n">
         <v>551</v>
@@ -20044,10 +20044,10 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>38.9</v>
+        <v>56.7</v>
       </c>
       <c r="G134" t="n">
-        <v>82.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="H134" t="n">
         <v>701</v>
@@ -20109,10 +20109,10 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>25.4</v>
+        <v>48.9</v>
       </c>
       <c r="G135" t="n">
-        <v>78.5</v>
+        <v>72.3</v>
       </c>
       <c r="H135" t="n">
         <v>853</v>
@@ -20174,10 +20174,10 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>46.1</v>
+        <v>60.8</v>
       </c>
       <c r="G136" t="n">
-        <v>87.5</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H136" t="n">
         <v>350</v>
@@ -20239,10 +20239,10 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>41</v>
+        <v>57.8</v>
       </c>
       <c r="G137" t="n">
-        <v>78</v>
+        <v>71.5</v>
       </c>
       <c r="H137" t="n">
         <v>455</v>
@@ -20304,10 +20304,10 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>62.9</v>
+        <v>70.3</v>
       </c>
       <c r="G138" t="n">
-        <v>74.90000000000001</v>
+        <v>67</v>
       </c>
       <c r="H138" t="n">
         <v>376</v>
@@ -20369,10 +20369,10 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>59.2</v>
+        <v>68.3</v>
       </c>
       <c r="G139" t="n">
-        <v>76.2</v>
+        <v>69</v>
       </c>
       <c r="H139" t="n">
         <v>507</v>
@@ -20434,10 +20434,10 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="G140" t="n">
-        <v>78.40000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="H140" t="n">
         <v>270</v>
@@ -20499,10 +20499,10 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>68.59999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G141" t="n">
-        <v>70.09999999999999</v>
+        <v>60</v>
       </c>
       <c r="H141" t="n">
         <v>242</v>

</xml_diff>